<commit_message>
updating final-output.py to most recent and minor changes to fs_app.py to support it
</commit_message>
<xml_diff>
--- a/formatted_output.xlsx
+++ b/formatted_output.xlsx
@@ -17,10 +17,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="$   #,##0;($   #,##0)"/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* (#,##0)"/>
     <numFmt numFmtId="165" formatCode="#,##0;(#,##0)"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,19 +29,49 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <color rgb="000000FF"/>
+      <name val="Helvetica Neue"/>
+      <sz val="8"/>
     </font>
     <font>
+      <name val="Helvetica Neue"/>
+      <color rgb="000070c0"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Helvetica Neue"/>
       <i val="1"/>
       <color rgb="00FF0000"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Helvetica Neue"/>
+      <sz val="24"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Helvetica Neue"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000000"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -56,27 +86,30 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="3"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -442,408 +475,435 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B4:D37"/>
+  <dimension ref="B1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>COMPANY NAME</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Consolidated Income Statements</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>2024</v>
+      </c>
+    </row>
     <row r="4">
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>ASSETS</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Current assets:</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Cash and cash equivalents</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="8" t="n">
         <v>73387</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="8" t="n">
         <v>78779</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Marketable securities</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="9" t="n">
         <v>13393</v>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D7" s="9" t="n">
         <v>22423</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Inventories</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="9" t="n">
         <v>33318</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="9" t="n">
         <v>34214</v>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Accounts receivable, net and other</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="9" t="n">
         <v>52253</v>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="D9" s="9" t="n">
         <v>55451</v>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Total current assets</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C10" s="9" t="n">
         <v>172351</v>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="D10" s="9" t="n">
         <v>190867</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Property and equipment, net</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C11" s="9" t="n">
         <v>204177</v>
       </c>
-      <c r="D11" s="6" t="n">
+      <c r="D11" s="9" t="n">
         <v>252665</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Operating leases</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="9" t="n">
         <v>72513</v>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="9" t="n">
         <v>76141</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Goodwill</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C13" s="9" t="n">
         <v>22789</v>
       </c>
-      <c r="D13" s="6" t="n">
+      <c r="D13" s="9" t="n">
         <v>23074</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Other assets</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C14" s="9" t="n">
         <v>56024</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D14" s="9" t="n">
         <v>82147</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Total assets</t>
         </is>
       </c>
-      <c r="C15" s="5" t="n">
+      <c r="C15" s="8" t="n">
         <v>527854</v>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D15" s="8" t="n">
         <v>624894</v>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="1" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>LIABILITIES AND STOCKHOLDERS EQUITY</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
+      <c r="C16" s="5" t="inlineStr"/>
+      <c r="D16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Current liabilities:</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr"/>
-      <c r="D17" s="2" t="inlineStr"/>
+      <c r="C17" s="5" t="inlineStr"/>
+      <c r="D17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Accounts payable</t>
         </is>
       </c>
-      <c r="C18" s="5" t="n">
+      <c r="C18" s="8" t="n">
         <v>84981</v>
       </c>
-      <c r="D18" s="5" t="n">
+      <c r="D18" s="8" t="n">
         <v>94363</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Accrued expenses and other</t>
         </is>
       </c>
-      <c r="C19" s="6" t="n">
+      <c r="C19" s="9" t="n">
         <v>64709</v>
       </c>
-      <c r="D19" s="6" t="n">
+      <c r="D19" s="9" t="n">
         <v>66965</v>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Unearned revenue</t>
         </is>
       </c>
-      <c r="C20" s="6" t="n">
+      <c r="C20" s="9" t="n">
         <v>15227</v>
       </c>
-      <c r="D20" s="6" t="n">
+      <c r="D20" s="9" t="n">
         <v>18103</v>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Total current liabilities</t>
         </is>
       </c>
-      <c r="C21" s="6" t="n">
+      <c r="C21" s="9" t="n">
         <v>164917</v>
       </c>
-      <c r="D21" s="6" t="n">
+      <c r="D21" s="9" t="n">
         <v>179431</v>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Long-term lease liabilities</t>
         </is>
       </c>
-      <c r="C22" s="6" t="n">
+      <c r="C22" s="9" t="n">
         <v>77297</v>
       </c>
-      <c r="D22" s="6" t="n">
+      <c r="D22" s="9" t="n">
         <v>78277</v>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>Long-term debt</t>
         </is>
       </c>
-      <c r="C23" s="6" t="n">
+      <c r="C23" s="9" t="n">
         <v>58314</v>
       </c>
-      <c r="D23" s="6" t="n">
+      <c r="D23" s="9" t="n">
         <v>52623</v>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Other long-term liabilities</t>
         </is>
       </c>
-      <c r="C24" s="6" t="n">
+      <c r="C24" s="9" t="n">
         <v>25451</v>
       </c>
-      <c r="D24" s="6" t="n">
+      <c r="D24" s="9" t="n">
         <v>28593</v>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>Commitments and contingencies (Note 7)</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr"/>
-      <c r="D25" s="2" t="inlineStr"/>
+      <c r="C25" s="5" t="inlineStr"/>
+      <c r="D25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>Stockholders' equity:</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
+      <c r="C26" s="5" t="inlineStr"/>
+      <c r="D26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>Preferred stock ($0.01 par value; 500 shares authorized; no shares issued or outstanding)</t>
         </is>
       </c>
-      <c r="C27" s="6" t="n">
+      <c r="C27" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D27" s="6" t="n">
+      <c r="D27" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>Common stock (S0.01 par value; 100,000 shares authorized; 10,898 and 11,108 shares</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
+      <c r="C28" s="5" t="inlineStr"/>
+      <c r="D28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>issued; 10,383 and 10,593 shares outstanding)</t>
         </is>
       </c>
-      <c r="C29" s="6" t="n">
+      <c r="C29" s="9" t="n">
         <v>109</v>
       </c>
-      <c r="D29" s="6" t="n">
+      <c r="D29" s="9" t="n">
         <v>111</v>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>Treasury stock, at cost</t>
         </is>
       </c>
-      <c r="C30" s="6" t="n">
+      <c r="C30" s="9" t="n">
         <v>-7837</v>
       </c>
-      <c r="D30" s="6" t="n">
+      <c r="D30" s="9" t="n">
         <v>-7837</v>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>Additional paid-in capital</t>
         </is>
       </c>
-      <c r="C31" s="6" t="n">
+      <c r="C31" s="9" t="n">
         <v>99025</v>
       </c>
-      <c r="D31" s="6" t="n">
+      <c r="D31" s="9" t="n">
         <v>120864</v>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B32" s="7" t="inlineStr">
         <is>
           <t>Accumulated other comprehensive income (loss)</t>
         </is>
       </c>
-      <c r="C32" s="6" t="n">
+      <c r="C32" s="9" t="n">
         <v>-3040</v>
       </c>
-      <c r="D32" s="6" t="n">
+      <c r="D32" s="9" t="n">
         <v>-34</v>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>Retained earnings</t>
         </is>
       </c>
-      <c r="C33" s="6" t="n">
+      <c r="C33" s="9" t="n">
         <v>113618</v>
       </c>
-      <c r="D33" s="6" t="n">
+      <c r="D33" s="9" t="n">
         <v>172866</v>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="7" t="inlineStr">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>Total stockholders' equity</t>
         </is>
       </c>
-      <c r="C34" s="6" t="n">
+      <c r="C34" s="9" t="n">
         <v>201875</v>
       </c>
-      <c r="D34" s="6" t="n">
+      <c r="D34" s="9" t="n">
         <v>285970</v>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>Total liabilities and stockholders' equity</t>
         </is>
       </c>
-      <c r="C35" s="5" t="n">
+      <c r="C35" s="8" t="n">
         <v>527854</v>
       </c>
-      <c r="D35" s="5" t="n">
+      <c r="D35" s="8" t="n">
         <v>624894</v>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="9" t="inlineStr">
-        <is>
-          <t>check</t>
-        </is>
-      </c>
-      <c r="C37">
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>Balance Check</t>
+        </is>
+      </c>
+      <c r="C37" s="12">
         <f>C35 - C15</f>
         <v/>
       </c>
-      <c r="D37">
+      <c r="D37" s="12">
         <f>D35 - D15</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
minor bug in collecting fs_type fixed
</commit_message>
<xml_diff>
--- a/formatted_output.xlsx
+++ b/formatted_output.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BALANCE_SHEET" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -50,6 +50,7 @@
     </font>
     <font>
       <name val="Helvetica Neue"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
@@ -86,11 +87,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -498,412 +502,412 @@
     </row>
     <row r="3">
       <c r="B3" s="2" t="n"/>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="4" t="n">
         <v>2023</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" s="4" t="n">
         <v>2024</v>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>ASSETS</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
+      <c r="C4" s="6" t="inlineStr"/>
+      <c r="D4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Current assets:</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
+      <c r="C5" s="6" t="inlineStr"/>
+      <c r="D5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Cash and cash equivalents</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="9" t="n">
         <v>73387</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="9" t="n">
         <v>78779</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Marketable securities</t>
         </is>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="10" t="n">
         <v>13393</v>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="10" t="n">
         <v>22423</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Inventories</t>
         </is>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="10" t="n">
         <v>33318</v>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="10" t="n">
         <v>34214</v>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Accounts receivable, net and other</t>
         </is>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C9" s="10" t="n">
         <v>52253</v>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="10" t="n">
         <v>55451</v>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Total current assets</t>
         </is>
       </c>
-      <c r="C10" s="9" t="n">
+      <c r="C10" s="10" t="n">
         <v>172351</v>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="10" t="n">
         <v>190867</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Property and equipment, net</t>
         </is>
       </c>
-      <c r="C11" s="9" t="n">
+      <c r="C11" s="10" t="n">
         <v>204177</v>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="10" t="n">
         <v>252665</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Operating leases</t>
         </is>
       </c>
-      <c r="C12" s="9" t="n">
+      <c r="C12" s="10" t="n">
         <v>72513</v>
       </c>
-      <c r="D12" s="9" t="n">
+      <c r="D12" s="10" t="n">
         <v>76141</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Goodwill</t>
         </is>
       </c>
-      <c r="C13" s="9" t="n">
+      <c r="C13" s="10" t="n">
         <v>22789</v>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="10" t="n">
         <v>23074</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Other assets</t>
         </is>
       </c>
-      <c r="C14" s="9" t="n">
+      <c r="C14" s="10" t="n">
         <v>56024</v>
       </c>
-      <c r="D14" s="9" t="n">
+      <c r="D14" s="10" t="n">
         <v>82147</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Total assets</t>
         </is>
       </c>
-      <c r="C15" s="8" t="n">
+      <c r="C15" s="9" t="n">
         <v>527854</v>
       </c>
-      <c r="D15" s="8" t="n">
+      <c r="D15" s="9" t="n">
         <v>624894</v>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>LIABILITIES AND STOCKHOLDERS EQUITY</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr"/>
-      <c r="D16" s="5" t="inlineStr"/>
+      <c r="C16" s="6" t="inlineStr"/>
+      <c r="D16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Current liabilities:</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr"/>
-      <c r="D17" s="5" t="inlineStr"/>
+      <c r="C17" s="6" t="inlineStr"/>
+      <c r="D17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Accounts payable</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
+      <c r="C18" s="9" t="n">
         <v>84981</v>
       </c>
-      <c r="D18" s="8" t="n">
+      <c r="D18" s="9" t="n">
         <v>94363</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Accrued expenses and other</t>
         </is>
       </c>
-      <c r="C19" s="9" t="n">
+      <c r="C19" s="10" t="n">
         <v>64709</v>
       </c>
-      <c r="D19" s="9" t="n">
+      <c r="D19" s="10" t="n">
         <v>66965</v>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Unearned revenue</t>
         </is>
       </c>
-      <c r="C20" s="9" t="n">
+      <c r="C20" s="10" t="n">
         <v>15227</v>
       </c>
-      <c r="D20" s="9" t="n">
+      <c r="D20" s="10" t="n">
         <v>18103</v>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>Total current liabilities</t>
         </is>
       </c>
-      <c r="C21" s="9" t="n">
+      <c r="C21" s="10" t="n">
         <v>164917</v>
       </c>
-      <c r="D21" s="9" t="n">
+      <c r="D21" s="10" t="n">
         <v>179431</v>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Long-term lease liabilities</t>
         </is>
       </c>
-      <c r="C22" s="9" t="n">
+      <c r="C22" s="10" t="n">
         <v>77297</v>
       </c>
-      <c r="D22" s="9" t="n">
+      <c r="D22" s="10" t="n">
         <v>78277</v>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Long-term debt</t>
         </is>
       </c>
-      <c r="C23" s="9" t="n">
+      <c r="C23" s="10" t="n">
         <v>58314</v>
       </c>
-      <c r="D23" s="9" t="n">
+      <c r="D23" s="10" t="n">
         <v>52623</v>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Other long-term liabilities</t>
         </is>
       </c>
-      <c r="C24" s="9" t="n">
+      <c r="C24" s="10" t="n">
         <v>25451</v>
       </c>
-      <c r="D24" s="9" t="n">
+      <c r="D24" s="10" t="n">
         <v>28593</v>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>Commitments and contingencies (Note 7)</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr"/>
-      <c r="D25" s="5" t="inlineStr"/>
+      <c r="C25" s="6" t="inlineStr"/>
+      <c r="D25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>Stockholders' equity:</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr"/>
-      <c r="D26" s="5" t="inlineStr"/>
+      <c r="C26" s="6" t="inlineStr"/>
+      <c r="D26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>Preferred stock ($0.01 par value; 500 shares authorized; no shares issued or outstanding)</t>
         </is>
       </c>
-      <c r="C27" s="9" t="n">
+      <c r="C27" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="D27" s="9" t="n">
+      <c r="D27" s="10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="7" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>Common stock (S0.01 par value; 100,000 shares authorized; 10,898 and 11,108 shares</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr"/>
-      <c r="D28" s="5" t="inlineStr"/>
+      <c r="C28" s="6" t="inlineStr"/>
+      <c r="D28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>issued; 10,383 and 10,593 shares outstanding)</t>
         </is>
       </c>
-      <c r="C29" s="9" t="n">
+      <c r="C29" s="10" t="n">
         <v>109</v>
       </c>
-      <c r="D29" s="9" t="n">
+      <c r="D29" s="10" t="n">
         <v>111</v>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="7" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>Treasury stock, at cost</t>
         </is>
       </c>
-      <c r="C30" s="9" t="n">
+      <c r="C30" s="10" t="n">
         <v>-7837</v>
       </c>
-      <c r="D30" s="9" t="n">
+      <c r="D30" s="10" t="n">
         <v>-7837</v>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>Additional paid-in capital</t>
         </is>
       </c>
-      <c r="C31" s="9" t="n">
+      <c r="C31" s="10" t="n">
         <v>99025</v>
       </c>
-      <c r="D31" s="9" t="n">
+      <c r="D31" s="10" t="n">
         <v>120864</v>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="7" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>Accumulated other comprehensive income (loss)</t>
         </is>
       </c>
-      <c r="C32" s="9" t="n">
+      <c r="C32" s="10" t="n">
         <v>-3040</v>
       </c>
-      <c r="D32" s="9" t="n">
+      <c r="D32" s="10" t="n">
         <v>-34</v>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>Retained earnings</t>
         </is>
       </c>
-      <c r="C33" s="9" t="n">
+      <c r="C33" s="10" t="n">
         <v>113618</v>
       </c>
-      <c r="D33" s="9" t="n">
+      <c r="D33" s="10" t="n">
         <v>172866</v>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="10" t="inlineStr">
+      <c r="B34" s="11" t="inlineStr">
         <is>
           <t>Total stockholders' equity</t>
         </is>
       </c>
-      <c r="C34" s="9" t="n">
+      <c r="C34" s="10" t="n">
         <v>201875</v>
       </c>
-      <c r="D34" s="9" t="n">
+      <c r="D34" s="10" t="n">
         <v>285970</v>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="11" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>Total liabilities and stockholders' equity</t>
         </is>
       </c>
-      <c r="C35" s="8" t="n">
+      <c r="C35" s="9" t="n">
         <v>527854</v>
       </c>
-      <c r="D35" s="8" t="n">
+      <c r="D35" s="9" t="n">
         <v>624894</v>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="12" t="inlineStr">
+      <c r="B37" s="13" t="inlineStr">
         <is>
           <t>Balance Check</t>
         </is>
       </c>
-      <c r="C37" s="12">
+      <c r="C37" s="13">
         <f>C35 - C15</f>
         <v/>
       </c>
-      <c r="D37" s="12">
+      <c r="D37" s="13">
         <f>D35 - D15</f>
         <v/>
       </c>

</xml_diff>